<commit_message>
Update 00981A report 2026-03-20
</commit_message>
<xml_diff>
--- a/etf_data/49YTW_20260320.xlsx
+++ b/etf_data/49YTW_20260320.xlsx
@@ -12,9 +12,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="231">
-  <si>
-    <t xml:space="preserve">資料日期：115/03/19</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="232">
+  <si>
+    <t xml:space="preserve">資料日期：115/03/20</t>
   </si>
   <si>
     <t xml:space="preserve">基金資產</t>
@@ -23,19 +23,19 @@
     <t xml:space="preserve">淨資產</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 91,253,421,358</t>
+    <t xml:space="preserve">NTD 93,824,460,628</t>
   </si>
   <si>
     <t xml:space="preserve">流通在外單位數</t>
   </si>
   <si>
-    <t xml:space="preserve">4,348,709,000</t>
+    <t xml:space="preserve">4,470,709,000</t>
   </si>
   <si>
     <t xml:space="preserve">每單位淨值</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 20.98</t>
+    <t xml:space="preserve">NTD 20.99</t>
   </si>
   <si>
     <t xml:space="preserve">項目</t>
@@ -59,19 +59,19 @@
     <t xml:space="preserve">股票</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 87,497,505,260</t>
-  </si>
-  <si>
-    <t xml:space="preserve">95.88%</t>
+    <t xml:space="preserve">NTD 89,058,921,050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94.92%</t>
   </si>
   <si>
     <t xml:space="preserve">現金</t>
   </si>
   <si>
-    <t xml:space="preserve">NTD 3,269,050,980</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.58%</t>
+    <t xml:space="preserve">NTD 3,948,717,772</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.21%</t>
   </si>
   <si>
     <t xml:space="preserve">期貨保證金</t>
@@ -80,355 +80,376 @@
     <t xml:space="preserve">NTD 500,128,241</t>
   </si>
   <si>
+    <t xml:space="preserve">0.53%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">申贖應付款</t>
+  </si>
+  <si>
+    <t xml:space="preserve">應收付證券款</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NTD -2,501,642,979</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.67%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">股票代號</t>
+  </si>
+  <si>
+    <t xml:space="preserve">股票名稱</t>
+  </si>
+  <si>
+    <t xml:space="preserve">股數</t>
+  </si>
+  <si>
+    <t xml:space="preserve">持股權重</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2330</t>
+  </si>
+  <si>
+    <t xml:space="preserve">台積電</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,405,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.64%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2383</t>
+  </si>
+  <si>
+    <t xml:space="preserve">台光電</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,427,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.27%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2308</t>
+  </si>
+  <si>
+    <t xml:space="preserve">台達電</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,309,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.77%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">奇鋐</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,876,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.28%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2368</t>
+  </si>
+  <si>
+    <t xml:space="preserve">金像電</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,765,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.07%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6223</t>
+  </si>
+  <si>
+    <t xml:space="preserve">旺矽</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,366,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.62%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3653</t>
+  </si>
+  <si>
+    <t xml:space="preserve">健策</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,328,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.45%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">智邦</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,034,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.21%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3665</t>
+  </si>
+  <si>
+    <t xml:space="preserve">貿聯-KY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,525,848</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.91%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">欣興</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7,410,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.38%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5274</t>
+  </si>
+  <si>
+    <t xml:space="preserve">信驊</t>
+  </si>
+  <si>
+    <t xml:space="preserve">255,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.19%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2327</t>
+  </si>
+  <si>
+    <t xml:space="preserve">國巨*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10,703,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.09%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">南電</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,656,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.68%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2449</t>
+  </si>
+  <si>
+    <t xml:space="preserve">京元電子</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7,062,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.32%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6510</t>
+  </si>
+  <si>
+    <t xml:space="preserve">精測</t>
+  </si>
+  <si>
+    <t xml:space="preserve">590,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.26%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6515</t>
+  </si>
+  <si>
+    <t xml:space="preserve">穎崴</t>
+  </si>
+  <si>
+    <t xml:space="preserve">248,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3661</t>
+  </si>
+  <si>
+    <t xml:space="preserve">世芯-KY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">530,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.91%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8210</t>
+  </si>
+  <si>
+    <t xml:space="preserve">勤誠</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,621,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.58%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3711</t>
+  </si>
+  <si>
+    <t xml:space="preserve">日月光投控</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,258,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.56%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">富世達</t>
+  </si>
+  <si>
+    <t xml:space="preserve">682,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.45%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1303</t>
+  </si>
+  <si>
+    <t xml:space="preserve">南亞</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15,336,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.28%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3189</t>
+  </si>
+  <si>
+    <t xml:space="preserve">景碩</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,657,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.08%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6139</t>
+  </si>
+  <si>
+    <t xml:space="preserve">亞翔</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,704,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2454</t>
+  </si>
+  <si>
+    <t xml:space="preserve">聯發科</t>
+  </si>
+  <si>
+    <t xml:space="preserve">486,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.88%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6488</t>
+  </si>
+  <si>
+    <t xml:space="preserve">環球晶</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,700,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.85%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3443</t>
+  </si>
+  <si>
+    <t xml:space="preserve">創意</t>
+  </si>
+  <si>
+    <t xml:space="preserve">245,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.69%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">漢唐</t>
+  </si>
+  <si>
+    <t xml:space="preserve">573,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.57%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3211</t>
+  </si>
+  <si>
+    <t xml:space="preserve">順達</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,576,000</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.55%</t>
   </si>
   <si>
-    <t xml:space="preserve">申贖應付款</t>
-  </si>
-  <si>
-    <t xml:space="preserve">應收付證券款</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NTD -1,585,984,358</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-1.74%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">股票代號</t>
-  </si>
-  <si>
-    <t xml:space="preserve">股票名稱</t>
-  </si>
-  <si>
-    <t xml:space="preserve">股數</t>
-  </si>
-  <si>
-    <t xml:space="preserve">持股權重</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2330</t>
-  </si>
-  <si>
-    <t xml:space="preserve">台積電</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,271,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.66%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2383</t>
-  </si>
-  <si>
-    <t xml:space="preserve">台光電</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,427,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.69%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2308</t>
-  </si>
-  <si>
-    <t xml:space="preserve">台達電</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,309,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.87%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2368</t>
-  </si>
-  <si>
-    <t xml:space="preserve">金像電</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,600,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.17%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3017</t>
-  </si>
-  <si>
-    <t xml:space="preserve">奇鋐</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,572,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.68%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3653</t>
-  </si>
-  <si>
-    <t xml:space="preserve">健策</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,297,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.54%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6223</t>
-  </si>
-  <si>
-    <t xml:space="preserve">旺矽</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,366,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.49%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2345</t>
-  </si>
-  <si>
-    <t xml:space="preserve">智邦</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,034,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.29%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3037</t>
-  </si>
-  <si>
-    <t xml:space="preserve">欣興</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7,410,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.72%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3665</t>
-  </si>
-  <si>
-    <t xml:space="preserve">貿聯-KY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,362,848</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.45%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5274</t>
-  </si>
-  <si>
-    <t xml:space="preserve">信驊</t>
-  </si>
-  <si>
-    <t xml:space="preserve">255,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.37%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2327</t>
-  </si>
-  <si>
-    <t xml:space="preserve">國巨*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10,251,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.09%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8046</t>
-  </si>
-  <si>
-    <t xml:space="preserve">南電</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,656,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.86%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2449</t>
-  </si>
-  <si>
-    <t xml:space="preserve">京元電子</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7,062,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.45%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6510</t>
-  </si>
-  <si>
-    <t xml:space="preserve">精測</t>
-  </si>
-  <si>
-    <t xml:space="preserve">590,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.30%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3661</t>
-  </si>
-  <si>
-    <t xml:space="preserve">世芯-KY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">589,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.08%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6515</t>
-  </si>
-  <si>
-    <t xml:space="preserve">穎崴</t>
-  </si>
-  <si>
-    <t xml:space="preserve">248,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.96%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3711</t>
-  </si>
-  <si>
-    <t xml:space="preserve">日月光投控</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4,258,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.62%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8210</t>
-  </si>
-  <si>
-    <t xml:space="preserve">勤誠</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,621,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.58%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">富世達</t>
-  </si>
-  <si>
-    <t xml:space="preserve">682,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.48%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1303</t>
-  </si>
-  <si>
-    <t xml:space="preserve">南亞</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15,336,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.42%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3189</t>
-  </si>
-  <si>
-    <t xml:space="preserve">景碩</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,657,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.12%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6139</t>
-  </si>
-  <si>
-    <t xml:space="preserve">亞翔</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,704,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.10%</t>
-  </si>
-  <si>
     <t xml:space="preserve">6274</t>
   </si>
   <si>
     <t xml:space="preserve">台燿</t>
   </si>
   <si>
-    <t xml:space="preserve">1,463,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.94%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2454</t>
-  </si>
-  <si>
-    <t xml:space="preserve">聯發科</t>
-  </si>
-  <si>
-    <t xml:space="preserve">486,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.89%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6488</t>
-  </si>
-  <si>
-    <t xml:space="preserve">環球晶</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,700,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.88%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2404</t>
-  </si>
-  <si>
-    <t xml:space="preserve">漢唐</t>
-  </si>
-  <si>
-    <t xml:space="preserve">573,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.57%</t>
+    <t xml:space="preserve">844,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.50%</t>
   </si>
   <si>
     <t xml:space="preserve">8358</t>
@@ -440,16 +461,7 @@
     <t xml:space="preserve">1,864,000</t>
   </si>
   <si>
-    <t xml:space="preserve">3211</t>
-  </si>
-  <si>
-    <t xml:space="preserve">順達</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,576,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.52%</t>
+    <t xml:space="preserve">0.49%</t>
   </si>
   <si>
     <t xml:space="preserve">5347</t>
@@ -461,7 +473,19 @@
     <t xml:space="preserve">3,848,000</t>
   </si>
   <si>
-    <t xml:space="preserve">0.50%</t>
+    <t xml:space="preserve">0.48%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4979</t>
+  </si>
+  <si>
+    <t xml:space="preserve">華星光</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,036,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.45%</t>
   </si>
   <si>
     <t xml:space="preserve">1326</t>
@@ -473,19 +497,79 @@
     <t xml:space="preserve">8,827,000</t>
   </si>
   <si>
-    <t xml:space="preserve">0.45%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4979</t>
-  </si>
-  <si>
-    <t xml:space="preserve">華星光</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,036,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.44%</t>
+    <t xml:space="preserve">0.43%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6191</t>
+  </si>
+  <si>
+    <t xml:space="preserve">精成科</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,399,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.35%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3376</t>
+  </si>
+  <si>
+    <t xml:space="preserve">新日興</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,425,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.34%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2408</t>
+  </si>
+  <si>
+    <t xml:space="preserve">南亞科</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,305,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.33%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8996</t>
+  </si>
+  <si>
+    <t xml:space="preserve">高力</t>
+  </si>
+  <si>
+    <t xml:space="preserve">315,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.31%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6669</t>
+  </si>
+  <si>
+    <t xml:space="preserve">緯穎</t>
+  </si>
+  <si>
+    <t xml:space="preserve">73,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3264</t>
+  </si>
+  <si>
+    <t xml:space="preserve">欣銓</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,789,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.29%</t>
   </si>
   <si>
     <t xml:space="preserve">1802</t>
@@ -494,76 +578,10 @@
     <t xml:space="preserve">台玻</t>
   </si>
   <si>
-    <t xml:space="preserve">5,996,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.40%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2408</t>
-  </si>
-  <si>
-    <t xml:space="preserve">南亞科</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,305,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.37%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6191</t>
-  </si>
-  <si>
-    <t xml:space="preserve">精成科</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3,399,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.36%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3376</t>
-  </si>
-  <si>
-    <t xml:space="preserve">新日興</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,425,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8996</t>
-  </si>
-  <si>
-    <t xml:space="preserve">高力</t>
-  </si>
-  <si>
-    <t xml:space="preserve">315,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.33%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3264</t>
-  </si>
-  <si>
-    <t xml:space="preserve">欣銓</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,789,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.30%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6669</t>
-  </si>
-  <si>
-    <t xml:space="preserve">緯穎</t>
-  </si>
-  <si>
-    <t xml:space="preserve">73,000</t>
+    <t xml:space="preserve">3,885,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.24%</t>
   </si>
   <si>
     <t xml:space="preserve">3533</t>
@@ -587,7 +605,7 @@
     <t xml:space="preserve">158,000</t>
   </si>
   <si>
-    <t xml:space="preserve">0.19%</t>
+    <t xml:space="preserve">0.18%</t>
   </si>
   <si>
     <t xml:space="preserve">1319</t>
@@ -638,61 +656,46 @@
     <t xml:space="preserve">0.02%</t>
   </si>
   <si>
-    <t xml:space="preserve">2059</t>
-  </si>
-  <si>
-    <t xml:space="preserve">川湖</t>
+    <t xml:space="preserve">2357</t>
+  </si>
+  <si>
+    <t xml:space="preserve">華碩</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.00%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1815</t>
+  </si>
+  <si>
+    <t xml:space="preserve">富喬</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2439</t>
+  </si>
+  <si>
+    <t xml:space="preserve">美律</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">台灣大</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5536</t>
+  </si>
+  <si>
+    <t xml:space="preserve">聖暉*</t>
   </si>
   <si>
     <t xml:space="preserve">4,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2357</t>
-  </si>
-  <si>
-    <t xml:space="preserve">華碩</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.00%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1815</t>
-  </si>
-  <si>
-    <t xml:space="preserve">富喬</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2439</t>
-  </si>
-  <si>
-    <t xml:space="preserve">美律</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8299</t>
-  </si>
-  <si>
-    <t xml:space="preserve">群聯</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">台灣大</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5536</t>
-  </si>
-  <si>
-    <t xml:space="preserve">聖暉*</t>
   </si>
   <si>
     <t xml:space="preserve">2313</t>
@@ -783,7 +786,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="247">
+  <cellXfs count="243">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="center" vertical="center"/>
@@ -865,18 +868,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1529,7 +1520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.9" bestFit="1" customWidth="1" collapsed="1"/>
@@ -2006,77 +1997,77 @@
         <v>121</v>
       </c>
       <c r="D43" s="122" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="123" t="s">
+        <v>122</v>
+      </c>
+      <c r="B44" s="124" t="s">
         <v>123</v>
       </c>
-      <c r="B44" s="124" t="s">
+      <c r="C44" s="125" t="s">
         <v>124</v>
       </c>
-      <c r="C44" s="125" t="s">
+      <c r="D44" s="126" t="s">
         <v>125</v>
-      </c>
-      <c r="D44" s="126" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="127" t="s">
+        <v>126</v>
+      </c>
+      <c r="B45" s="128" t="s">
         <v>127</v>
       </c>
-      <c r="B45" s="128" t="s">
+      <c r="C45" s="129" t="s">
         <v>128</v>
       </c>
-      <c r="C45" s="129" t="s">
+      <c r="D45" s="130" t="s">
         <v>129</v>
-      </c>
-      <c r="D45" s="130" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="131" t="s">
+        <v>130</v>
+      </c>
+      <c r="B46" s="132" t="s">
         <v>131</v>
       </c>
-      <c r="B46" s="132" t="s">
+      <c r="C46" s="133" t="s">
         <v>132</v>
       </c>
-      <c r="C46" s="133" t="s">
+      <c r="D46" s="134" t="s">
         <v>133</v>
-      </c>
-      <c r="D46" s="134" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="135" t="s">
+        <v>134</v>
+      </c>
+      <c r="B47" s="136" t="s">
         <v>135</v>
       </c>
-      <c r="B47" s="136" t="s">
+      <c r="C47" s="137" t="s">
         <v>136</v>
       </c>
-      <c r="C47" s="137" t="s">
+      <c r="D47" s="138" t="s">
         <v>137</v>
-      </c>
-      <c r="D47" s="138" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="139" t="s">
+        <v>138</v>
+      </c>
+      <c r="B48" s="140" t="s">
         <v>139</v>
       </c>
-      <c r="B48" s="140" t="s">
+      <c r="C48" s="141" t="s">
         <v>140</v>
       </c>
-      <c r="C48" s="141" t="s">
+      <c r="D48" s="142" t="s">
         <v>141</v>
-      </c>
-      <c r="D48" s="142" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="49">
@@ -2188,259 +2179,245 @@
         <v>172</v>
       </c>
       <c r="D56" s="174" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="175" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B57" s="176" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C57" s="177" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D57" s="178" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="179" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B58" s="180" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C58" s="181" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D58" s="182" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="183" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B59" s="184" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C59" s="185" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D59" s="186" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="187" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B60" s="188" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C60" s="189" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D60" s="190" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="191" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B61" s="192" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C61" s="193" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D61" s="194" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="195" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B62" s="196" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C62" s="197" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D62" s="198" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="199" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B63" s="200" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C63" s="201" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D63" s="202" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="203" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B64" s="204" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C64" s="205" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D64" s="206" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="207" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B65" s="208" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C65" s="209" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D65" s="210" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="211" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B66" s="212" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C66" s="213" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D66" s="214" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="215" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B67" s="216" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C67" s="217" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D67" s="218" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="219" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B68" s="220" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="C68" s="221" t="s">
+        <v>220</v>
+      </c>
+      <c r="D68" s="222" t="s">
         <v>217</v>
-      </c>
-      <c r="D68" s="222" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="223" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B69" s="224" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C69" s="225" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="D69" s="226" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="227" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B70" s="228" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C70" s="229" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="D70" s="230" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="231" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B71" s="232" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C71" s="233" t="s">
-        <v>213</v>
+        <v>227</v>
       </c>
       <c r="D71" s="234" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="235" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B72" s="236" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C72" s="237" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="D72" s="238" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="239" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B73" s="240" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="C73" s="241" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="D73" s="242" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="243" t="s">
-        <v>229</v>
-      </c>
-      <c r="B74" s="244" t="s">
-        <v>230</v>
-      </c>
-      <c r="C74" s="245" t="s">
-        <v>213</v>
-      </c>
-      <c r="D74" s="246" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>